<commit_message>
Update product prototypes and PRDs across risk control, customs, FCL, and commission modules.
Includes查货操作 fee modal, QUICK_FEE remarks, notification list, and PRD sidebar cleanup.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/报关行对接/报关系统场景.xlsx
+++ b/报关行对接/报关系统场景.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12375"/>
+    <workbookView windowWidth="28800" windowHeight="12255"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="场景合并" sheetId="1" r:id="rId1"/>
+    <sheet name="报关系统场景" sheetId="2" r:id="rId2"/>
+    <sheet name="报关行场景" sheetId="3" r:id="rId3"/>
+    <sheet name="报关行场景原图" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,40 +30,54 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>场景</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="44">
+  <si>
+    <t>来源</t>
+  </si>
+  <si>
+    <t>场景分类</t>
+  </si>
+  <si>
+    <t>子场景</t>
+  </si>
+  <si>
+    <t>场景描述</t>
+  </si>
+  <si>
+    <t>方案</t>
+  </si>
+  <si>
+    <t>优先级/备注</t>
+  </si>
+  <si>
+    <t>报关系统</t>
+  </si>
+  <si>
+    <t>报关资料制作</t>
   </si>
   <si>
     <t>客户初次报关，或对报关资料制作不熟练</t>
   </si>
   <si>
-    <r>
-      <t>例如：客户初次</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">制作报关资料不熟练，推送后问题过多，会进行多次沟通修改或多次重新上传报关资料，是否会按照原单号覆盖。
-</t>
-    </r>
+    <t>例如：客户初次制作报关资料不熟练，推送后问题过多，会进行多次沟通修改或多次重新上传报关资料，是否会按照原单号覆盖。</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>分单号绑定</t>
   </si>
   <si>
     <t>原先漏勾选报关，绑定分单号后勾选</t>
   </si>
   <si>
-    <t>在绑定分单号后，会有客户漏勾选报关，上传了资料，询问后才进行勾选，需增加一票报关</t>
+    <t>在绑定分单号后，会有客户漏勾选报关，上传了资料，询问后才进行勾选，需增加一票报关。</t>
   </si>
   <si>
     <t>改买单</t>
   </si>
   <si>
-    <t>例：因客观原因，原本打算报关客户，需改为买单出，后这个单号依旧存在，但是不能用这个客户的抬头报了（分单号不变，但是实际内容需要进行变更，不能再使用原先预录单）</t>
+    <t>例：因客观原因，原本打算报关客户，需改为买单出，后这个单号依旧存在，但是不能用这个客户的抬头报了（分单号不变，但是实际内容需要进行变更，不能再使用原先预录单）。</t>
   </si>
   <si>
     <t>测试出现问题</t>
@@ -71,14 +86,82 @@
     <t>沟通困难</t>
   </si>
   <si>
-    <t xml:space="preserve">例1：绑定分单号与客户知道的单号不一致，发过去客户会有疑惑，或者觉得不是自己的不认同       例2：因需要改名发客户，与报关行沟通又出现问题，容易出现沟通错误。
-</t>
+    <t>例1：绑定分单号与客户知道的单号不一致，发过去客户会有疑惑，或者觉得不是自己的不认同。例2：因需要改名发客户，与报关行沟通又出现问题，容易出现沟通错误。</t>
   </si>
   <si>
     <t>下载文件重复</t>
   </si>
   <si>
-    <t>预录单修改后会有多份预录单，不便寻找</t>
+    <t>预录单修改后会有多份预录单，不便寻找。</t>
+  </si>
+  <si>
+    <t>报关行</t>
+  </si>
+  <si>
+    <t>签入或终配舱报关单号推送</t>
+  </si>
+  <si>
+    <t>客户合并报关正确</t>
+  </si>
+  <si>
+    <t>报关单号推送；报关单号抓取资料。</t>
+  </si>
+  <si>
+    <t>客户合并报关调整</t>
+  </si>
+  <si>
+    <t>例如：123一单、456一单已推送；调整为1245一单、36一单。前面的两单需要跟报关行沟通作废（申报之前）；将新的重新推送过去，我们系统以新的为准。</t>
+  </si>
+  <si>
+    <t>优</t>
+  </si>
+  <si>
+    <t>客户合并报关需要拆</t>
+  </si>
+  <si>
+    <t>例如：123456一单已推送；调整为1245一单、36一单。前面的一单需要跟报关行沟通作废（申报之前）；将新的重新推送过去，我们系统以新的为准。</t>
+  </si>
+  <si>
+    <t>配仓减少</t>
+  </si>
+  <si>
+    <t>例如：12、34、56三单已推送；调整为56删除。56的一单需要跟报关行沟通作废；其他不影响。</t>
+  </si>
+  <si>
+    <t>配仓增加</t>
+  </si>
+  <si>
+    <t>例如：12、34、56三单已推送；新增78增加；78重新推送；其他不影响。</t>
+  </si>
+  <si>
+    <t>分单号推送</t>
+  </si>
+  <si>
+    <t>分单号录入正确</t>
+  </si>
+  <si>
+    <t>分单号推送；分单号抓取资料。</t>
+  </si>
+  <si>
+    <t>分单号录入错误</t>
+  </si>
+  <si>
+    <t>分单号推送；分单号修改推送；分单号抓取资料。</t>
+  </si>
+  <si>
+    <t>已拦截。例如：123一单、456一单已推送；调整为1245一单、36一单。需要修改分单号重新推送，原单作废。</t>
+  </si>
+  <si>
+    <t>例如：123456一单拆分为2单；绑定分单号的时候分为1245一单、36一单推送；以我们系统推送的为准。</t>
+  </si>
+  <si>
+    <t>已拦截。例如：12、34、56三单已推送；调整为56删除。56的分单号需要沿用，会被报关行拦截；分单号需要调整重推，前面的全部作废。</t>
+  </si>
+  <si>
+    <t>例如：12、34、56三单已推送；新增78；78重新推送；其他不影响。</t>
+  </si>
+  <si>
+    <t>报关行场景（原 PNG 对照）</t>
   </si>
 </sst>
 </file>
@@ -91,7 +174,29 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,20 +348,19 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -553,166 +657,160 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -766,7 +864,7 @@
     <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -775,10 +873,46 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7381875" cy="6438900"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="352425"/>
+          <a:ext cx="7381875" cy="6438900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="WPS">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -786,39 +920,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4874CB"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="EE822F"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="F2BA02"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="75BD42"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="30C0B4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="E54C5E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0026E5"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="7E1FAD"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="WPS">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -850,7 +984,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -885,135 +1018,171 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="WPS">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumOff val="17500"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
-              <a:schemeClr val="phClr"/>
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="2700000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:hueOff val="-2520000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
-              <a:schemeClr val="phClr"/>
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="2700000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:gradFill>
-            <a:gsLst>
-              <a:gs pos="0">
-                <a:schemeClr val="phClr">
-                  <a:hueOff val="-4200000"/>
-                </a:schemeClr>
-              </a:gs>
-              <a:gs pos="100000">
-                <a:schemeClr val="phClr"/>
-              </a:gs>
-            </a:gsLst>
-            <a:lin ang="2700000" scaled="1"/>
-          </a:gradFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="101600" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:schemeClr val="phClr">
-                <a:alpha val="60000"/>
-              </a:schemeClr>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:reflection stA="50000" endA="300" endPos="40000" dist="25400" dir="5400000" sy="-100000" algn="bl" rotWithShape="0"/>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
           </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1025,66 +1194,325 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="2"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="23.875" customWidth="1"/>
-    <col min="2" max="2" width="33.75" customWidth="1"/>
-    <col min="3" max="3" width="29.25" customWidth="1"/>
-    <col min="8" max="8" width="7.125" customWidth="1"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="5" width="72" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" ht="109" customHeight="1" spans="1:3">
-      <c r="B2" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" ht="40.5" spans="1:3">
-      <c r="B3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" ht="81" spans="1:3">
-      <c r="B4" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="2" ht="72" customHeight="1" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1" spans="1:6">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1" spans="1:6">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" ht="94.5" spans="1:3">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" ht="27" spans="1:3">
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>11</v>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1" spans="1:6">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1" spans="1:6">
+      <c r="A8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1" spans="1:6">
+      <c r="A9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1" spans="1:6">
+      <c r="A10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1" spans="1:6">
+      <c r="A11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1" spans="1:6">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1" spans="1:6">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1" spans="1:6">
+      <c r="A14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1" spans="1:6">
+      <c r="A15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1" spans="1:6">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1" spans="1:6">
+      <c r="A17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -1092,11 +1520,119 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1" spans="1:5">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1" spans="1:5">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1" spans="1:5">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1" spans="1:5">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1" spans="1:5">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -1104,11 +1640,242 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1" spans="1:5">
+      <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1" spans="1:5">
+      <c r="A3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1" spans="1:5">
+      <c r="A4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1" spans="1:5">
+      <c r="A5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1" spans="1:5">
+      <c r="A6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1" spans="1:5">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1" spans="1:5">
+      <c r="A8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1" spans="1:5">
+      <c r="A9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1" spans="1:5">
+      <c r="A10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1" spans="1:5">
+      <c r="A11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1" spans="1:5">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="14.25" spans="1:1">
+      <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>